<commit_message>
Add geschaeftsreise: Rückflug Madrid - Augsburg (Team Global Tech Innovations)
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -94,7 +94,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -105,7 +105,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,6 +124,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -492,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -587,7 +590,7 @@
           <t>Flugrechnung</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="11" t="n"/>
       <c r="E2" s="5" t="n">
         <v>0</v>
       </c>
@@ -602,10 +605,10 @@
           <t>Spanien</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="11" t="n">
         <v>46305</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="11" t="n">
         <v>46305</v>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -619,61 +622,91 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Flugticket-Rueckflug-Madrid-Augsburg.md</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Rückflug Madrid - Augsburg (Team Global Tech Innovations)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Flugticket</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="n"/>
+      <c r="E3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>46310</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Ticketbeleg für den Rückflug des 10-köpfigen Teams von Madrid über München nach Augsburg am 15. Oktober 2026, inkl. Rail&amp;Fly-Verbindung mit dem ICE.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="9">
-        <f>SUM(E2:E2)</f>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="9">
+        <f>SUM(E2:E3)</f>
         <v/>
       </c>
-      <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8" t="n"/>
-      <c r="K4" s="8" t="n"/>
-      <c r="L4" s="8" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="n"/>
+      <c r="L5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A6" s="3" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
@@ -687,18 +720,15 @@
       <c r="L6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
-      <c r="E7" s="5">
-        <f>SUMIF(C2:C2,A7,E2:E2)</f>
-        <v/>
-      </c>
+      <c r="E7" s="6" t="n"/>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
@@ -707,10 +737,53 @@
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Flugrechnung</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="5">
+        <f>SUMIF(C2:C3,A8,E2:E3)</f>
+        <v/>
+      </c>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Flugticket</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="5">
+        <f>SUMIF(C2:C3,A9,E2:E3)</f>
+        <v/>
+      </c>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:L3"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Uber Business Sammelabrechnung Madrid
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -670,61 +670,91 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Taxi-Uber-Sammelabrechnung.md</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Uber Business Sammelabrechnung Madrid</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>46309</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Sammelabrechnung für Uber-Fahrten (Uber Comfort/Black/Van) während der Geschäftsreise nach Madrid vom 10. bis 14. Oktober 2026, insgesamt drei Fahrten zwischen Flughafen, Hotel, Business Park und Dinner Event.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="9">
-        <f>SUM(E2:E3)</f>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="9">
+        <f>SUM(E2:E4)</f>
         <v/>
       </c>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="8" t="n"/>
+      <c r="K6" s="8" t="n"/>
+      <c r="L6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
@@ -738,18 +768,15 @@
       <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
-      <c r="E8" s="5">
-        <f>SUMIF(C2:C3,A8,E2:E3)</f>
-        <v/>
-      </c>
+      <c r="E8" s="6" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
@@ -761,14 +788,14 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="5">
-        <f>SUMIF(C2:C3,A9,E2:E3)</f>
+        <f>SUMIF(C2:C4,A9,E2:E4)</f>
         <v/>
       </c>
       <c r="F9" s="3" t="n"/>
@@ -779,11 +806,54 @@
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Flugticket</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="5">
+        <f>SUMIF(C2:C4,A10,E2:E4)</f>
+        <v/>
+      </c>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="5">
+        <f>SUMIF(C2:C4,A11,E2:E4)</f>
+        <v/>
+      </c>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L3"/>
+  <autoFilter ref="A1:L4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Workshop- & Eventrechnung Tech Strategy & Innovation Summit Madrid 2026
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -718,61 +718,91 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Workshop-Madrid-Summit.md</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Workshop- &amp; Eventrechnung Tech Strategy &amp; Innovation Summit Madrid 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Rechnung für einen zweitägigen Workshop im Rahmen des Tech Strategy &amp; Innovation Summit in Madrid, veranstaltet von Madrid Executive Innovation Hub S.L. im Impact Hub Madrid - Gobernador. Enthält Kosten für Raummiete, Moderation und Catering.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="9">
-        <f>SUM(E2:E4)</f>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="9">
+        <f>SUM(E2:E5)</f>
         <v/>
       </c>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
@@ -786,18 +816,15 @@
       <c r="L8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
-      <c r="E9" s="5">
-        <f>SUMIF(C2:C4,A9,E2:E4)</f>
-        <v/>
-      </c>
+      <c r="E9" s="6" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
@@ -809,14 +836,14 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="5">
-        <f>SUMIF(C2:C4,A10,E2:E4)</f>
+        <f>SUMIF(C2:C5,A10,E2:E5)</f>
         <v/>
       </c>
       <c r="F10" s="3" t="n"/>
@@ -830,14 +857,14 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="5">
-        <f>SUMIF(C2:C4,A11,E2:E4)</f>
+        <f>SUMIF(C2:C5,A11,E2:E5)</f>
         <v/>
       </c>
       <c r="F11" s="3" t="n"/>
@@ -848,12 +875,55 @@
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="5">
+        <f>SUMIF(C2:C5,A12,E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="5">
+        <f>SUMIF(C2:C5,A13,E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L4"/>
+  <autoFilter ref="A1:L5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Parkgebühren Tiefgarage Plaza de España Madrid
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -766,61 +766,91 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Parkhaus-Quittung-Madrid.md</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Parkgebühren Tiefgarage Plaza de España Madrid</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Parkticket</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>46310</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Quittung für Langzeit-Parkticket in der Tiefgarage Plaza de España, Madrid, für 2 Mietwagen der Firmen-Delegation über 5 Tage (10.10.–15.10.2026).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="9">
-        <f>SUM(E2:E5)</f>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="9">
+        <f>SUM(E2:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
+      <c r="L8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
@@ -834,18 +864,15 @@
       <c r="L9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
-      <c r="E10" s="5">
-        <f>SUMIF(C2:C5,A10,E2:E5)</f>
-        <v/>
-      </c>
+      <c r="E10" s="6" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
@@ -857,14 +884,14 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="5">
-        <f>SUMIF(C2:C5,A11,E2:E5)</f>
+        <f>SUMIF(C2:C6,A11,E2:E6)</f>
         <v/>
       </c>
       <c r="F11" s="3" t="n"/>
@@ -878,14 +905,14 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="5">
-        <f>SUMIF(C2:C5,A12,E2:E5)</f>
+        <f>SUMIF(C2:C6,A12,E2:E6)</f>
         <v/>
       </c>
       <c r="F12" s="3" t="n"/>
@@ -899,14 +926,14 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Taxi</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="5">
-        <f>SUMIF(C2:C5,A13,E2:E5)</f>
+        <f>SUMIF(C2:C6,A13,E2:E6)</f>
         <v/>
       </c>
       <c r="F13" s="3" t="n"/>
@@ -917,13 +944,56 @@
       <c r="K13" s="3" t="n"/>
       <c r="L13" s="3" t="n"/>
     </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="5">
+        <f>SUMIF(C2:C6,A14,E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Parkticket</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="5">
+        <f>SUMIF(C2:C6,A15,E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: ÖPNV Quittung Metro Madrid
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -814,61 +814,91 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>OePNV-Metro-Madrid.md</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ÖPNV Quittung Metro Madrid</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="5" t="n">
+        <v>251</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Beleg über den Kauf von 10 Tourist-Pässen (5-Tage, Zone A) für die Nutzung des öffentlichen Nahverkehrs in Madrid inklusive Multi-Card.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="9">
-        <f>SUM(E2:E6)</f>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="9">
+        <f>SUM(E2:E7)</f>
         <v/>
       </c>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="8" t="n"/>
+      <c r="L9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
@@ -882,18 +912,15 @@
       <c r="L10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
-      <c r="E11" s="5">
-        <f>SUMIF(C2:C6,A11,E2:E6)</f>
-        <v/>
-      </c>
+      <c r="E11" s="6" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
@@ -905,14 +932,14 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="5">
-        <f>SUMIF(C2:C6,A12,E2:E6)</f>
+        <f>SUMIF(C2:C7,A12,E2:E7)</f>
         <v/>
       </c>
       <c r="F12" s="3" t="n"/>
@@ -926,14 +953,14 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="5">
-        <f>SUMIF(C2:C6,A13,E2:E6)</f>
+        <f>SUMIF(C2:C7,A13,E2:E7)</f>
         <v/>
       </c>
       <c r="F13" s="3" t="n"/>
@@ -947,14 +974,14 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Taxi</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="5">
-        <f>SUMIF(C2:C6,A14,E2:E6)</f>
+        <f>SUMIF(C2:C7,A14,E2:E7)</f>
         <v/>
       </c>
       <c r="F14" s="3" t="n"/>
@@ -968,14 +995,14 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Parkticket</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="5">
-        <f>SUMIF(C2:C6,A15,E2:E6)</f>
+        <f>SUMIF(C2:C7,A15,E2:E7)</f>
         <v/>
       </c>
       <c r="F15" s="3" t="n"/>
@@ -986,14 +1013,57 @@
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Parkticket</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="5">
+        <f>SUMIF(C2:C7,A16,E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="5">
+        <f>SUMIF(C2:C7,A17,E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L7"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Minibar Eigenbeleg Hotel Riu Plaza España Madrid
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -862,61 +862,91 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Minibar-Rechnung-Madrid.md</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Minibar Eigenbeleg Hotel Riu Plaza España Madrid</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>46310</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Eigenbeleg für Minibar-Konsum der Zimmer 401 bis 410 (Team Global Tech) im Hotel Riu Plaza España, Madrid, über Hotelrechnung beglichen.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="9">
-        <f>SUM(E2:E7)</f>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="9">
+        <f>SUM(E2:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="8" t="n"/>
-      <c r="L9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="8" t="n"/>
+      <c r="K10" s="8" t="n"/>
+      <c r="L10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
@@ -930,18 +960,15 @@
       <c r="L11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
-      <c r="E12" s="5">
-        <f>SUMIF(C2:C7,A12,E2:E7)</f>
-        <v/>
-      </c>
+      <c r="E12" s="6" t="n"/>
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n"/>
@@ -953,14 +980,14 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="5">
-        <f>SUMIF(C2:C7,A13,E2:E7)</f>
+        <f>SUMIF(C2:C8,A13,E2:E8)</f>
         <v/>
       </c>
       <c r="F13" s="3" t="n"/>
@@ -974,14 +1001,14 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="5">
-        <f>SUMIF(C2:C7,A14,E2:E7)</f>
+        <f>SUMIF(C2:C8,A14,E2:E8)</f>
         <v/>
       </c>
       <c r="F14" s="3" t="n"/>
@@ -995,14 +1022,14 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Taxi</t>
         </is>
       </c>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="5">
-        <f>SUMIF(C2:C7,A15,E2:E7)</f>
+        <f>SUMIF(C2:C8,A15,E2:E8)</f>
         <v/>
       </c>
       <c r="F15" s="3" t="n"/>
@@ -1016,14 +1043,14 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Parkticket</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="5">
-        <f>SUMIF(C2:C7,A16,E2:E7)</f>
+        <f>SUMIF(C2:C8,A16,E2:E8)</f>
         <v/>
       </c>
       <c r="F16" s="3" t="n"/>
@@ -1037,14 +1064,14 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Sonstiges</t>
+          <t>Parkticket</t>
         </is>
       </c>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="5">
-        <f>SUMIF(C2:C7,A17,E2:E7)</f>
+        <f>SUMIF(C2:C8,A17,E2:E8)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="n"/>
@@ -1055,8 +1082,29 @@
       <c r="K17" s="3" t="n"/>
       <c r="L17" s="3" t="n"/>
     </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="5">
+        <f>SUMIF(C2:C8,A18,E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:L8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -1064,6 +1112,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Mietwagenrechnung Sixt Madrid
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -910,61 +910,91 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Mietwagen-Sixt-Madrid.md</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Mietwagenrechnung Sixt Madrid</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Mietwagen</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="5" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>46310</v>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Rechnung von Sixt Autovermietung für die Anmietung von 2x Premium Minivan (BMW X5 / Mercedes V-Klasse) an der Station Madrid Barajas Airport T4 für den Zeitraum 10.10.2026 bis 15.10.2026.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="9">
-        <f>SUM(E2:E8)</f>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="9">
+        <f>SUM(E2:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
-      <c r="L10" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="8" t="n"/>
+      <c r="K11" s="8" t="n"/>
+      <c r="L11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
@@ -978,18 +1008,15 @@
       <c r="L12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
-      <c r="E13" s="5">
-        <f>SUMIF(C2:C8,A13,E2:E8)</f>
-        <v/>
-      </c>
+      <c r="E13" s="6" t="n"/>
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="n"/>
@@ -1001,14 +1028,14 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="5">
-        <f>SUMIF(C2:C8,A14,E2:E8)</f>
+        <f>SUMIF(C2:C9,A14,E2:E9)</f>
         <v/>
       </c>
       <c r="F14" s="3" t="n"/>
@@ -1022,14 +1049,14 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="5">
-        <f>SUMIF(C2:C8,A15,E2:E8)</f>
+        <f>SUMIF(C2:C9,A15,E2:E9)</f>
         <v/>
       </c>
       <c r="F15" s="3" t="n"/>
@@ -1043,14 +1070,14 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Taxi</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="5">
-        <f>SUMIF(C2:C8,A16,E2:E8)</f>
+        <f>SUMIF(C2:C9,A16,E2:E9)</f>
         <v/>
       </c>
       <c r="F16" s="3" t="n"/>
@@ -1064,14 +1091,14 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Parkticket</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="5">
-        <f>SUMIF(C2:C8,A17,E2:E8)</f>
+        <f>SUMIF(C2:C9,A17,E2:E9)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="n"/>
@@ -1085,14 +1112,14 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Sonstiges</t>
+          <t>Parkticket</t>
         </is>
       </c>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="5">
-        <f>SUMIF(C2:C8,A18,E2:E8)</f>
+        <f>SUMIF(C2:C9,A18,E2:E9)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="n"/>
@@ -1103,8 +1130,50 @@
       <c r="K18" s="3" t="n"/>
       <c r="L18" s="3" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="5">
+        <f>SUMIF(C2:C9,A19,E2:E9)</f>
+        <v/>
+      </c>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Mietwagen</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="5">
+        <f>SUMIF(C2:C9,A20,E2:E9)</f>
+        <v/>
+      </c>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:L9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -1113,6 +1182,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Hotelrechnung Riu Plaza España Madrid
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -958,61 +958,91 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Hotelrechnung-Riu-Plaza-Espana.md</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung Riu Plaza España Madrid</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="5" t="n">
+        <v>7900</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>46310</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung des Hotels Riu Plaza España in Madrid für 10 Zimmer über 5 Nächte im Rahmen einer Geschäftsreise der Global Tech Innovations GmbH.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="9">
-        <f>SUM(E2:E9)</f>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="9">
+        <f>SUM(E2:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="8" t="n"/>
-      <c r="L11" s="8" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
+      <c r="J12" s="8" t="n"/>
+      <c r="K12" s="8" t="n"/>
+      <c r="L12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
@@ -1026,18 +1056,15 @@
       <c r="L13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
-      <c r="E14" s="5">
-        <f>SUMIF(C2:C9,A14,E2:E9)</f>
-        <v/>
-      </c>
+      <c r="E14" s="6" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
@@ -1049,14 +1076,14 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="5">
-        <f>SUMIF(C2:C9,A15,E2:E9)</f>
+        <f>SUMIF(C2:C10,A15,E2:E10)</f>
         <v/>
       </c>
       <c r="F15" s="3" t="n"/>
@@ -1070,14 +1097,14 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="5">
-        <f>SUMIF(C2:C9,A16,E2:E9)</f>
+        <f>SUMIF(C2:C10,A16,E2:E10)</f>
         <v/>
       </c>
       <c r="F16" s="3" t="n"/>
@@ -1091,14 +1118,14 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Taxi</t>
         </is>
       </c>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="5">
-        <f>SUMIF(C2:C9,A17,E2:E9)</f>
+        <f>SUMIF(C2:C10,A17,E2:E10)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="n"/>
@@ -1112,14 +1139,14 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Parkticket</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="5">
-        <f>SUMIF(C2:C9,A18,E2:E9)</f>
+        <f>SUMIF(C2:C10,A18,E2:E10)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="n"/>
@@ -1133,14 +1160,14 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Sonstiges</t>
+          <t>Parkticket</t>
         </is>
       </c>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="5">
-        <f>SUMIF(C2:C9,A19,E2:E9)</f>
+        <f>SUMIF(C2:C10,A19,E2:E10)</f>
         <v/>
       </c>
       <c r="F19" s="3" t="n"/>
@@ -1154,14 +1181,14 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Mietwagen</t>
+          <t>Sonstiges</t>
         </is>
       </c>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="5">
-        <f>SUMIF(C2:C9,A20,E2:E9)</f>
+        <f>SUMIF(C2:C10,A20,E2:E10)</f>
         <v/>
       </c>
       <c r="F20" s="3" t="n"/>
@@ -1172,8 +1199,50 @@
       <c r="K20" s="3" t="n"/>
       <c r="L20" s="3" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Mietwagen</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="5">
+        <f>SUMIF(C2:C10,A21,E2:E10)</f>
+        <v/>
+      </c>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="5">
+        <f>SUMIF(C2:C10,A22,E2:E10)</f>
+        <v/>
+      </c>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:L10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -1183,6 +1252,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Bewirtungsbeleg Restaurante Botín Madrid
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1006,61 +1006,91 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg-Restaurante-Botin.md</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg Restaurante Botín Madrid</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>46305</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>46307</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg für ein Geschäftsessen mit 10 Teilnehmern im Restaurante Botín in Madrid im Rahmen eines Partner-Meetings zur Besprechung der Expansionsstrategie Iberia.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="9">
-        <f>SUM(E2:E10)</f>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="9">
+        <f>SUM(E2:E11)</f>
         <v/>
       </c>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
-      <c r="L12" s="8" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="8" t="n"/>
+      <c r="K13" s="8" t="n"/>
+      <c r="L13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
@@ -1074,18 +1104,15 @@
       <c r="L14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
-      <c r="E15" s="5">
-        <f>SUMIF(C2:C10,A15,E2:E10)</f>
-        <v/>
-      </c>
+      <c r="E15" s="6" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
@@ -1097,14 +1124,14 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="5">
-        <f>SUMIF(C2:C10,A16,E2:E10)</f>
+        <f>SUMIF(C2:C11,A16,E2:E11)</f>
         <v/>
       </c>
       <c r="F16" s="3" t="n"/>
@@ -1118,14 +1145,14 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="5">
-        <f>SUMIF(C2:C10,A17,E2:E10)</f>
+        <f>SUMIF(C2:C11,A17,E2:E11)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="n"/>
@@ -1139,14 +1166,14 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Taxi</t>
         </is>
       </c>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="5">
-        <f>SUMIF(C2:C10,A18,E2:E10)</f>
+        <f>SUMIF(C2:C11,A18,E2:E11)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="n"/>
@@ -1160,14 +1187,14 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Parkticket</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="5">
-        <f>SUMIF(C2:C10,A19,E2:E10)</f>
+        <f>SUMIF(C2:C11,A19,E2:E11)</f>
         <v/>
       </c>
       <c r="F19" s="3" t="n"/>
@@ -1181,14 +1208,14 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Sonstiges</t>
+          <t>Parkticket</t>
         </is>
       </c>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="5">
-        <f>SUMIF(C2:C10,A20,E2:E10)</f>
+        <f>SUMIF(C2:C11,A20,E2:E11)</f>
         <v/>
       </c>
       <c r="F20" s="3" t="n"/>
@@ -1202,14 +1229,14 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Mietwagen</t>
+          <t>Sonstiges</t>
         </is>
       </c>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="5">
-        <f>SUMIF(C2:C10,A21,E2:E10)</f>
+        <f>SUMIF(C2:C11,A21,E2:E11)</f>
         <v/>
       </c>
       <c r="F21" s="3" t="n"/>
@@ -1223,14 +1250,14 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Hotelrechnung</t>
+          <t>Mietwagen</t>
         </is>
       </c>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="5">
-        <f>SUMIF(C2:C10,A22,E2:E10)</f>
+        <f>SUMIF(C2:C11,A22,E2:E11)</f>
         <v/>
       </c>
       <c r="F22" s="3" t="n"/>
@@ -1241,8 +1268,50 @@
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
     </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Hotelrechnung</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="5">
+        <f>SUMIF(C2:C11,A23,E2:E11)</f>
+        <v/>
+      </c>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="5">
+        <f>SUMIF(C2:C11,A24,E2:E11)</f>
+        <v/>
+      </c>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L10"/>
+  <autoFilter ref="A1:L11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -1253,6 +1322,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Renfe Bahntickets Madrid-Toledo Tagesausflug
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reiseübersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reiseübersicht'!$A$1:$L$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1054,61 +1054,91 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Bahnticket-Renfe-Toledo.md</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Renfe Bahntickets Madrid-Toledo Tagesausflug</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Bahnticket</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="5" t="n">
+        <v>278</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>46308</v>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Gruppenbahntickets für einen Tagesausflug von Madrid nach Toledo und zurück am 13.10.2026 im Rahmen der Geschäftsreise nach Madrid.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Gesamtkosten</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="9">
-        <f>SUM(E2:E11)</f>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="9">
+        <f>SUM(E2:E12)</f>
         <v/>
       </c>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="8" t="n"/>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="8" t="n"/>
+      <c r="K14" s="8" t="n"/>
+      <c r="L14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
+      <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
@@ -1122,18 +1152,15 @@
       <c r="L15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Flugrechnung</t>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
-      <c r="E16" s="5">
-        <f>SUMIF(C2:C11,A16,E2:E11)</f>
-        <v/>
-      </c>
+      <c r="E16" s="6" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n"/>
@@ -1145,14 +1172,14 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Flugticket</t>
+          <t>Flugrechnung</t>
         </is>
       </c>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="5">
-        <f>SUMIF(C2:C11,A17,E2:E11)</f>
+        <f>SUMIF(C2:C12,A17,E2:E12)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="n"/>
@@ -1166,14 +1193,14 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Taxi</t>
+          <t>Flugticket</t>
         </is>
       </c>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="5">
-        <f>SUMIF(C2:C11,A18,E2:E11)</f>
+        <f>SUMIF(C2:C12,A18,E2:E12)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="n"/>
@@ -1187,14 +1214,14 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Taxi</t>
         </is>
       </c>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="5">
-        <f>SUMIF(C2:C11,A19,E2:E11)</f>
+        <f>SUMIF(C2:C12,A19,E2:E12)</f>
         <v/>
       </c>
       <c r="F19" s="3" t="n"/>
@@ -1208,14 +1235,14 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Parkticket</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="5">
-        <f>SUMIF(C2:C11,A20,E2:E11)</f>
+        <f>SUMIF(C2:C12,A20,E2:E12)</f>
         <v/>
       </c>
       <c r="F20" s="3" t="n"/>
@@ -1229,14 +1256,14 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Sonstiges</t>
+          <t>Parkticket</t>
         </is>
       </c>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="5">
-        <f>SUMIF(C2:C11,A21,E2:E11)</f>
+        <f>SUMIF(C2:C12,A21,E2:E12)</f>
         <v/>
       </c>
       <c r="F21" s="3" t="n"/>
@@ -1250,14 +1277,14 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Mietwagen</t>
+          <t>Sonstiges</t>
         </is>
       </c>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="5">
-        <f>SUMIF(C2:C11,A22,E2:E11)</f>
+        <f>SUMIF(C2:C12,A22,E2:E12)</f>
         <v/>
       </c>
       <c r="F22" s="3" t="n"/>
@@ -1271,14 +1298,14 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Hotelrechnung</t>
+          <t>Mietwagen</t>
         </is>
       </c>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="5">
-        <f>SUMIF(C2:C11,A23,E2:E11)</f>
+        <f>SUMIF(C2:C12,A23,E2:E12)</f>
         <v/>
       </c>
       <c r="F23" s="3" t="n"/>
@@ -1292,14 +1319,14 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Bewirtungsbeleg</t>
+          <t>Hotelrechnung</t>
         </is>
       </c>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="3" t="n"/>
       <c r="E24" s="5">
-        <f>SUMIF(C2:C11,A24,E2:E11)</f>
+        <f>SUMIF(C2:C12,A24,E2:E12)</f>
         <v/>
       </c>
       <c r="F24" s="3" t="n"/>
@@ -1310,8 +1337,50 @@
       <c r="K24" s="3" t="n"/>
       <c r="L24" s="3" t="n"/>
     </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Bewirtungsbeleg</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="5">
+        <f>SUMIF(C2:C12,A25,E2:E12)</f>
+        <v/>
+      </c>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Bahnticket</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="5">
+        <f>SUMIF(C2:C12,A26,E2:E12)</f>
+        <v/>
+      </c>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -1323,6 +1392,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add geschaeftsreise: Renfe Bahntickets Madrid - Toledo Tagesausflug
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q4/2026-10-10_Madrid/Reiseübersicht.xlsx
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -1062,7 +1061,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Renfe Bahntickets Madrid-Toledo Tagesausflug</t>
+          <t>Renfe Bahntickets Madrid - Toledo Tagesausflug</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1098,7 +1097,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>Gruppenbahntickets für einen Tagesausflug von Madrid nach Toledo und zurück am 13.10.2026 im Rahmen der Geschäftsreise nach Madrid.</t>
+          <t>Gruppenbahntickets für einen Tagesausflug von Madrid nach Toledo und zurück im Rahmen der Geschäftsreise nach Madrid.</t>
         </is>
       </c>
     </row>

</xml_diff>